<commit_message>
fix: correct Calu-3 and nasal cell ontology terms
Co-authored-by: sierra-moxon <4561292+sierra-moxon@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/src/docs/Liu2024_PM25_CFTR_SOMA.xlsx
+++ b/src/docs/Liu2024_PM25_CFTR_SOMA.xlsx
@@ -1,28 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protocol" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ExposureCondition" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KeyEvent" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CellularSystem" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="InVivoSubject" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CFTRFunctionAssay" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CFTRFunctionOutput" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GeneExpressionAssay" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GeneExpressionOutput" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GobletCellAssay" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GobletCellOutput" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BALFSputumAssay" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BALFSputumOutput" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LungFunctionAssay" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LungFunctionOutput" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Metadata" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Protocol" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="ExposureCondition" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="KeyEvent" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="CellularSystem" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="InVivoSubject" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="CFTRFunctionAssay" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="CFTRFunctionOutput" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="GeneExpressionAssay" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="GeneExpressionOutput" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="GobletCellAssay" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="GobletCellOutput" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="BALFSputumAssay" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="BALFSputumOutput" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="LungFunctionAssay" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="LungFunctionOutput" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -757,7 +757,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>UO:0000193</t>
+          <t>fold change (UO:0000193)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr"/>
@@ -789,7 +789,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>UO:0000193</t>
+          <t>fold change (UO:0000193)</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr"/>
@@ -823,7 +823,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>UO:0000193</t>
+          <t>fold change (UO:0000193)</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -855,7 +855,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>UO:0000193</t>
+          <t>fold change (UO:0000193)</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -889,7 +889,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>UO:0000187</t>
+          <t>percent (UO:0000187)</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>UO:0000187</t>
+          <t>percent (UO:0000187)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr"/>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>UO:0000187</t>
+          <t>percent (UO:0000187)</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr"/>
@@ -1434,7 +1434,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>UO:0000193</t>
+          <t>fold change vs OVA (UO:0000193)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1676,7 +1676,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>UO:0000193</t>
+          <t>fold change vs control (UO:0000193)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1704,7 +1704,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>UO:0000193</t>
+          <t>fold change vs control (UO:0000193)</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -2077,7 +2077,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>CHEBI:74481</t>
+          <t>ENVO:01000415</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -2087,7 +2087,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>UO:0000064</t>
+          <t>ug/mL (UO:0000064)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -2097,7 +2097,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>UO:0000032</t>
+          <t>hour (UO:0000032)</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>CHEBI:74481</t>
+          <t>ENVO:01000415</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -2129,7 +2129,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>UO:0000064</t>
+          <t>ug/mL (UO:0000064)</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>UO:0000032</t>
+          <t>hour (UO:0000032)</t>
         </is>
       </c>
     </row>
@@ -2161,7 +2161,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>CHEBI:74481</t>
+          <t>ENVO:01000415</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -2171,7 +2171,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>UO:0000064</t>
+          <t>ug/mL (UO:0000064)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -2181,7 +2181,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>UO:0000033</t>
+          <t>day (UO:0000033)</t>
         </is>
       </c>
     </row>
@@ -2213,7 +2213,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>UO:0000308</t>
+          <t>mg/kg (UO:0000308)</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -2223,7 +2223,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>UO:0000033</t>
+          <t>day (UO:0000033)</t>
         </is>
       </c>
     </row>
@@ -2245,7 +2245,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>CHEBI:45653</t>
+          <t>CHEBI:45906</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -2255,7 +2255,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>UO:0000308</t>
+          <t>mg/kg (UO:0000308)</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -2265,7 +2265,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>UO:0000033</t>
+          <t>day (UO:0000033)</t>
         </is>
       </c>
     </row>
@@ -2596,7 +2596,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>CLO:0003679</t>
+          <t>CLO:0002192</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
@@ -2771,7 +2771,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>UO:0000034</t>
+          <t>week (UO:0000034)</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -2830,7 +2830,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>UO:0000034</t>
+          <t>week (UO:0000034)</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -2897,7 +2897,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>UO:0000034</t>
+          <t>week (UO:0000034)</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -2960,7 +2960,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>UO:0000034</t>
+          <t>week (UO:0000034)</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -3346,7 +3346,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>UO:0000193</t>
+          <t>fold change (UO:0000193)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr"/>
@@ -3378,7 +3378,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>UO:0000193</t>
+          <t>fold change (UO:0000193)</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr"/>
@@ -3410,7 +3410,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>UO:0000193</t>
+          <t>fold change (UO:0000193)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr"/>
@@ -3442,7 +3442,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>UO:0000193</t>
+          <t>fold change (UO:0000193)</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr"/>

</xml_diff>